<commit_message>
changed value from 5% to 8%
</commit_message>
<xml_diff>
--- a/SuppXLS/Scen_Peak_RSV.xlsx
+++ b/SuppXLS/Scen_Peak_RSV.xlsx
@@ -1,6 +1,6 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" mc:Ignorable="x15 xr xr6 xr10">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" mc:Ignorable="x15 xr xr6 xr10">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="22730"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
@@ -8,13 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\VEDA\Training material\DemoS_012\SuppXLS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{73E9F4C3-E512-45C8-B41C-90BFA8E3A1FA}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1905" yWindow="1905" windowWidth="21600" windowHeight="11385"/>
+    <workbookView xWindow="1905" yWindow="1905" windowWidth="21600" windowHeight="11385" activeTab="0"/>
   </bookViews>
   <sheets>
-    <sheet name="Peak_RSV" sheetId="2" r:id="rId1"/>
+    <sheet name="Peak_RSV" sheetId="2" r:id="rId3"/>
   </sheets>
+  <definedNames/>
   <calcPr calcId="125725"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -28,19 +28,18 @@
 </file>
 
 <file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
   <authors>
     <author>Maurizio Gargiulo</author>
     <author>Gary Goldstein</author>
   </authors>
   <commentList>
-    <comment ref="B2" authorId="0" shapeId="0">
+    <comment ref="B2" authorId="0">
       <text>
         <r>
           <rPr>
             <b/>
             <sz val="8"/>
-            <color indexed="81"/>
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
@@ -48,12 +47,11 @@
         </r>
       </text>
     </comment>
-    <comment ref="J2" authorId="1" shapeId="0">
+    <comment ref="J2" authorId="1">
       <text>
         <r>
           <rPr>
             <sz val="8"/>
-            <color indexed="81"/>
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
@@ -61,12 +59,11 @@
         </r>
       </text>
     </comment>
-    <comment ref="O2" authorId="1" shapeId="0">
+    <comment ref="O2" authorId="1">
       <text>
         <r>
           <rPr>
             <sz val="8"/>
-            <color indexed="81"/>
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
@@ -81,80 +78,86 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="21">
   <si>
+    <t>Val_Cond</t>
+  </si>
+  <si>
+    <t>Cset_Set</t>
+  </si>
+  <si>
+    <t>REG1</t>
+  </si>
+  <si>
+    <t>Pset_Set</t>
+  </si>
+  <si>
+    <t>Attribute</t>
+  </si>
+  <si>
+    <t>Attrib_Cond</t>
+  </si>
+  <si>
+    <t>Cset_CN</t>
+  </si>
+  <si>
+    <t>Cset_CD</t>
+  </si>
+  <si>
+    <t>ELC</t>
+  </si>
+  <si>
+    <t>COM_PEAK</t>
+  </si>
+  <si>
+    <t>Pset_PD</t>
+  </si>
+  <si>
+    <t>AllRegions</t>
+  </si>
+  <si>
+    <t>Year</t>
+  </si>
+  <si>
+    <t>LimType</t>
+  </si>
+  <si>
+    <t>Pset_CO</t>
+  </si>
+  <si>
     <t>Pset_CI</t>
   </si>
   <si>
-    <t>Year</t>
+    <t>COM_PKRSV</t>
+  </si>
+  <si>
+    <t>~TFM_INS</t>
+  </si>
+  <si>
+    <t>Trans - Insert</t>
+  </si>
+  <si>
+    <t>TimeSlice</t>
   </si>
   <si>
     <t>Pset_PN</t>
-  </si>
-  <si>
-    <t>Pset_Set</t>
-  </si>
-  <si>
-    <t>Cset_CN</t>
-  </si>
-  <si>
-    <t>Pset_CO</t>
-  </si>
-  <si>
-    <t>Attribute</t>
-  </si>
-  <si>
-    <t>LimType</t>
-  </si>
-  <si>
-    <t>~TFM_INS</t>
-  </si>
-  <si>
-    <t>TimeSlice</t>
-  </si>
-  <si>
-    <t>AllRegions</t>
-  </si>
-  <si>
-    <t>Pset_PD</t>
-  </si>
-  <si>
-    <t>Cset_Set</t>
-  </si>
-  <si>
-    <t>Cset_CD</t>
-  </si>
-  <si>
-    <t>Attrib_Cond</t>
-  </si>
-  <si>
-    <t>Val_Cond</t>
-  </si>
-  <si>
-    <t>Trans - Insert</t>
-  </si>
-  <si>
-    <t>COM_PKRSV</t>
-  </si>
-  <si>
-    <t>ELC</t>
-  </si>
-  <si>
-    <t>COM_PEAK</t>
-  </si>
-  <si>
-    <t>REG1</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="8" x14ac:knownFonts="1">
+  <fonts count="8">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="11"/>
@@ -183,22 +186,13 @@
     <font>
       <b/>
       <sz val="8"/>
-      <color indexed="81"/>
       <name val="Tahoma"/>
       <family val="2"/>
     </font>
     <font>
       <sz val="8"/>
-      <color indexed="81"/>
       <name val="Tahoma"/>
       <family val="2"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="4">
@@ -233,46 +227,152 @@
       <left/>
       <right/>
       <top style="thin">
-        <color indexed="64"/>
+        <color auto="1"/>
       </top>
       <bottom style="medium">
-        <color indexed="64"/>
+        <color auto="1"/>
       </bottom>
-      <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="4">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
-    <xf numFmtId="9" fontId="7" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+  <cellStyleXfs count="22">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
+      <alignment/>
+      <protection/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="41" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0">
+      <alignment/>
+      <protection/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0">
+      <alignment/>
+      <protection/>
+    </xf>
   </cellStyleXfs>
   <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFill="1"/>
-    <xf numFmtId="2" fontId="3" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1"/>
-    <xf numFmtId="9" fontId="3" fillId="0" borderId="0" xfId="3" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="20" applyFill="1">
+      <alignment/>
+      <protection/>
+    </xf>
+    <xf numFmtId="2" fontId="4" fillId="0" borderId="0" xfId="20" applyNumberFormat="1" applyFill="1">
+      <alignment/>
+      <protection/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="20">
+      <alignment/>
+      <protection/>
+    </xf>
+    <xf numFmtId="9" fontId="4" fillId="0" borderId="0" xfId="15" applyFont="1" applyFill="1"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
-  <cellStyles count="4">
+  <cellStyles count="8">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Normal 10" xfId="1"/>
-    <cellStyle name="Normale_Scen_UC_IND-StrucConst" xfId="2"/>
-    <cellStyle name="Percent" xfId="3" builtinId="5"/>
+    <cellStyle name="Percent" xfId="15" builtinId="5"/>
+    <cellStyle name="Currency" xfId="16" builtinId="4"/>
+    <cellStyle name="Currency [0]" xfId="17" builtinId="7"/>
+    <cellStyle name="Comma" xfId="18" builtinId="3"/>
+    <cellStyle name="Comma [0]" xfId="19" builtinId="6"/>
+    <cellStyle name="Normal 10" xfId="20"/>
+    <cellStyle name="Normale_Scen_UC_IND-StrucConst" xfId="21"/>
   </cellStyles>
-  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -285,7 +385,7 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>1</xdr:col>
@@ -299,12 +399,12 @@
       <xdr:row>11</xdr:row>
       <xdr:rowOff>9525</xdr:rowOff>
     </xdr:to>
-    <xdr:sp macro="" textlink="">
+    <xdr:sp>
       <xdr:nvSpPr>
         <xdr:cNvPr id="3" name="TextBox 2">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D4D9DE9A-4331-4877-A0B6-2DA5742008B6}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{d4d9de9a-4331-4877-a0b6-2da5742008b6}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -312,12 +412,10 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="609601" y="1533525"/>
+          <a:off x="609600" y="1533525"/>
           <a:ext cx="5562600" cy="581025"/>
         </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
+        <a:prstGeom prst="rect"/>
         <a:solidFill>
           <a:schemeClr val="accent6">
             <a:lumMod val="20000"/>
@@ -326,7 +424,7 @@
         </a:solidFill>
         <a:ln w="9525" cmpd="sng">
           <a:solidFill>
-            <a:schemeClr val="lt1">
+            <a:schemeClr val="bg1">
               <a:shade val="50000"/>
             </a:schemeClr>
           </a:solidFill>
@@ -334,16 +432,16 @@
       </xdr:spPr>
       <xdr:style>
         <a:lnRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
+          <a:srgbClr val="000000"/>
         </a:lnRef>
         <a:fillRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
+          <a:srgbClr val="000000"/>
         </a:fillRef>
         <a:effectRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
+          <a:srgbClr val="000000"/>
         </a:effectRef>
         <a:fontRef idx="minor">
-          <a:schemeClr val="dk1"/>
+          <a:schemeClr val="tx1"/>
         </a:fontRef>
       </xdr:style>
       <xdr:txBody>
@@ -354,7 +452,7 @@
           <a:r>
             <a:rPr lang="en-GB" sz="1100">
               <a:solidFill>
-                <a:schemeClr val="dk1"/>
+                <a:schemeClr val="tx1"/>
               </a:solidFill>
               <a:effectLst/>
               <a:latin typeface="+mn-lt"/>
@@ -369,7 +467,7 @@
           <a:r>
             <a:rPr lang="en-GB" sz="1100">
               <a:solidFill>
-                <a:schemeClr val="dk1"/>
+                <a:schemeClr val="tx1"/>
               </a:solidFill>
               <a:effectLst/>
               <a:latin typeface="+mn-lt"/>
@@ -383,7 +481,7 @@
           <a:pPr lvl="0"/>
           <a:endParaRPr lang="en-GB" sz="1100">
             <a:solidFill>
-              <a:schemeClr val="dk1"/>
+              <a:schemeClr val="tx1"/>
             </a:solidFill>
             <a:effectLst/>
             <a:latin typeface="+mn-lt"/>
@@ -718,34 +816,34 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:Q9"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" width="10.140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="8.85546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="12.7109375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="5.140625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="9.7109375" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.7109375" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="10.7109375" customWidth="1"/>
-    <col min="10" max="10" width="8.7109375" bestFit="1" customWidth="1"/>
-    <col min="11" max="12" width="8.42578125" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="7.5703125" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="8.5703125" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="8.7109375" bestFit="1" customWidth="1"/>
-    <col min="16" max="17" width="8.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.1428571428571" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="8.85714285714286" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12.7142857142857" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="5.14285714285714" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11.5714285714286" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="9.71428571428571" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="10.7142857142857" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="10.7142857142857" customWidth="1"/>
+    <col min="10" max="10" width="8.71428571428571" bestFit="1" customWidth="1"/>
+    <col min="11" max="12" width="8.42857142857143" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="7.57142857142857" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="8.57142857142857" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="8.71428571428571" bestFit="1" customWidth="1"/>
+    <col min="16" max="17" width="8.42857142857143" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:1" ht="15">
       <c r="A1" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
     </row>
-    <row r="2" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="2" spans="2:17" ht="15">
       <c r="B2" s="1" t="s">
-        <v>8</v>
+        <v>17</v>
       </c>
       <c r="J2" s="2"/>
       <c r="K2" s="3"/>
@@ -756,106 +854,106 @@
       <c r="P2" s="3"/>
       <c r="Q2" s="3"/>
     </row>
-    <row r="3" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="2:17" ht="15.75" thickBot="1">
       <c r="B3" s="4" t="s">
-        <v>9</v>
+        <v>19</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="F3" s="4" t="s">
-        <v>14</v>
+        <v>5</v>
       </c>
       <c r="G3" s="4" t="s">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="H3" s="5" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="I3" s="5" t="s">
-        <v>20</v>
+        <v>2</v>
       </c>
       <c r="J3" s="6" t="s">
         <v>3</v>
       </c>
       <c r="K3" s="6" t="s">
-        <v>2</v>
+        <v>20</v>
       </c>
       <c r="L3" s="6" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="M3" s="6" t="s">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="N3" s="6" t="s">
-        <v>5</v>
+        <v>14</v>
       </c>
       <c r="O3" s="6" t="s">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="P3" s="6" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="Q3" s="6" t="s">
-        <v>13</v>
+        <v>7</v>
       </c>
     </row>
-    <row r="4" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="4" spans="4:16" ht="15">
       <c r="D4" s="7" t="s">
-        <v>19</v>
+        <v>9</v>
       </c>
       <c r="I4" s="8">
         <v>1</v>
       </c>
       <c r="P4" t="s">
-        <v>18</v>
+        <v>8</v>
       </c>
     </row>
-    <row r="5" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="5" spans="4:16" ht="15">
       <c r="D5" s="7" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="E5">
         <v>2005</v>
       </c>
       <c r="I5" s="10">
-        <v>0.05</v>
+        <v>0.08</v>
       </c>
       <c r="P5" t="s">
-        <v>18</v>
+        <v>8</v>
       </c>
     </row>
-    <row r="6" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="6" spans="4:16" ht="15">
       <c r="D6" s="7" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="E6">
         <v>2020</v>
       </c>
       <c r="I6" s="11">
-        <v>0.2</v>
+        <v>0.20</v>
       </c>
       <c r="P6" t="s">
-        <v>18</v>
+        <v>8</v>
       </c>
     </row>
-    <row r="7" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="7" spans="4:9" ht="15">
       <c r="D7" s="7"/>
       <c r="I7" s="8"/>
     </row>
-    <row r="9" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="9" spans="5:8" ht="15">
       <c r="E9" s="7"/>
       <c r="H9" s="9"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId1"/>
-  <legacyDrawing r:id="rId2"/>
+  <drawing r:id="rId2"/>
+  <legacyDrawing r:id="rId3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Value changed to 5%
</commit_message>
<xml_diff>
--- a/SuppXLS/Scen_Peak_RSV.xlsx
+++ b/SuppXLS/Scen_Peak_RSV.xlsx
@@ -78,67 +78,67 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="21">
   <si>
+    <t>Pset_CI</t>
+  </si>
+  <si>
+    <t>Year</t>
+  </si>
+  <si>
+    <t>Pset_PN</t>
+  </si>
+  <si>
+    <t>Pset_Set</t>
+  </si>
+  <si>
+    <t>Cset_CN</t>
+  </si>
+  <si>
+    <t>Pset_CO</t>
+  </si>
+  <si>
+    <t>Attribute</t>
+  </si>
+  <si>
+    <t>LimType</t>
+  </si>
+  <si>
+    <t>Trans - Insert</t>
+  </si>
+  <si>
+    <t>TimeSlice</t>
+  </si>
+  <si>
+    <t>AllRegions</t>
+  </si>
+  <si>
+    <t>Pset_PD</t>
+  </si>
+  <si>
+    <t>Cset_Set</t>
+  </si>
+  <si>
+    <t>Cset_CD</t>
+  </si>
+  <si>
+    <t>Attrib_Cond</t>
+  </si>
+  <si>
     <t>Val_Cond</t>
   </si>
   <si>
-    <t>Cset_Set</t>
+    <t>~TFM_INS</t>
+  </si>
+  <si>
+    <t>ELC</t>
+  </si>
+  <si>
+    <t>COM_PKRSV</t>
+  </si>
+  <si>
+    <t>COM_PEAK</t>
   </si>
   <si>
     <t>REG1</t>
-  </si>
-  <si>
-    <t>Pset_Set</t>
-  </si>
-  <si>
-    <t>Attribute</t>
-  </si>
-  <si>
-    <t>Attrib_Cond</t>
-  </si>
-  <si>
-    <t>Cset_CN</t>
-  </si>
-  <si>
-    <t>Cset_CD</t>
-  </si>
-  <si>
-    <t>ELC</t>
-  </si>
-  <si>
-    <t>COM_PEAK</t>
-  </si>
-  <si>
-    <t>Pset_PD</t>
-  </si>
-  <si>
-    <t>AllRegions</t>
-  </si>
-  <si>
-    <t>Year</t>
-  </si>
-  <si>
-    <t>LimType</t>
-  </si>
-  <si>
-    <t>Pset_CO</t>
-  </si>
-  <si>
-    <t>Pset_CI</t>
-  </si>
-  <si>
-    <t>COM_PKRSV</t>
-  </si>
-  <si>
-    <t>~TFM_INS</t>
-  </si>
-  <si>
-    <t>Trans - Insert</t>
-  </si>
-  <si>
-    <t>TimeSlice</t>
-  </si>
-  <si>
-    <t>Pset_PN</t>
   </si>
 </sst>
 </file>
@@ -838,12 +838,12 @@
   <sheetData>
     <row r="1" spans="1:1" ht="15">
       <c r="A1" t="s">
-        <v>18</v>
+        <v>8</v>
       </c>
     </row>
     <row r="2" spans="2:17" ht="15">
       <c r="B2" s="1" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="J2" s="2"/>
       <c r="K2" s="3"/>
@@ -856,82 +856,82 @@
     </row>
     <row r="3" spans="2:17" ht="15.75" thickBot="1">
       <c r="B3" s="4" t="s">
-        <v>19</v>
+        <v>9</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="F3" s="4" t="s">
-        <v>5</v>
+        <v>14</v>
       </c>
       <c r="G3" s="4" t="s">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="H3" s="5" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="I3" s="5" t="s">
-        <v>2</v>
+        <v>20</v>
       </c>
       <c r="J3" s="6" t="s">
         <v>3</v>
       </c>
       <c r="K3" s="6" t="s">
-        <v>20</v>
+        <v>2</v>
       </c>
       <c r="L3" s="6" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="M3" s="6" t="s">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="N3" s="6" t="s">
-        <v>14</v>
+        <v>5</v>
       </c>
       <c r="O3" s="6" t="s">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="P3" s="6" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="Q3" s="6" t="s">
-        <v>7</v>
+        <v>13</v>
       </c>
     </row>
     <row r="4" spans="4:16" ht="15">
       <c r="D4" s="7" t="s">
-        <v>9</v>
+        <v>19</v>
       </c>
       <c r="I4" s="8">
         <v>1</v>
       </c>
       <c r="P4" t="s">
-        <v>8</v>
+        <v>17</v>
       </c>
     </row>
     <row r="5" spans="4:16" ht="15">
       <c r="D5" s="7" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="E5">
         <v>2005</v>
       </c>
       <c r="I5" s="10">
-        <v>0.08</v>
+        <v>0.05</v>
       </c>
       <c r="P5" t="s">
-        <v>8</v>
+        <v>17</v>
       </c>
     </row>
     <row r="6" spans="4:16" ht="15">
       <c r="D6" s="7" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="E6">
         <v>2020</v>
@@ -940,7 +940,7 @@
         <v>0.20</v>
       </c>
       <c r="P6" t="s">
-        <v>8</v>
+        <v>17</v>
       </c>
     </row>
     <row r="7" spans="4:9" ht="15">

</xml_diff>

<commit_message>
REG1 value changed from 20% to 20%
</commit_message>
<xml_diff>
--- a/SuppXLS/Scen_Peak_RSV.xlsx
+++ b/SuppXLS/Scen_Peak_RSV.xlsx
@@ -78,67 +78,67 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="21">
   <si>
+    <t>Val_Cond</t>
+  </si>
+  <si>
+    <t>Cset_Set</t>
+  </si>
+  <si>
+    <t>REG1</t>
+  </si>
+  <si>
+    <t>Pset_Set</t>
+  </si>
+  <si>
+    <t>Attribute</t>
+  </si>
+  <si>
+    <t>Attrib_Cond</t>
+  </si>
+  <si>
+    <t>Cset_CN</t>
+  </si>
+  <si>
+    <t>Cset_CD</t>
+  </si>
+  <si>
+    <t>ELC</t>
+  </si>
+  <si>
+    <t>COM_PEAK</t>
+  </si>
+  <si>
+    <t>Pset_PD</t>
+  </si>
+  <si>
+    <t>AllRegions</t>
+  </si>
+  <si>
+    <t>Year</t>
+  </si>
+  <si>
+    <t>LimType</t>
+  </si>
+  <si>
+    <t>Pset_CO</t>
+  </si>
+  <si>
     <t>Pset_CI</t>
   </si>
   <si>
-    <t>Year</t>
+    <t>COM_PKRSV</t>
+  </si>
+  <si>
+    <t>~TFM_INS</t>
+  </si>
+  <si>
+    <t>Trans - Insert</t>
+  </si>
+  <si>
+    <t>TimeSlice</t>
   </si>
   <si>
     <t>Pset_PN</t>
-  </si>
-  <si>
-    <t>Pset_Set</t>
-  </si>
-  <si>
-    <t>Cset_CN</t>
-  </si>
-  <si>
-    <t>Pset_CO</t>
-  </si>
-  <si>
-    <t>Attribute</t>
-  </si>
-  <si>
-    <t>LimType</t>
-  </si>
-  <si>
-    <t>Trans - Insert</t>
-  </si>
-  <si>
-    <t>TimeSlice</t>
-  </si>
-  <si>
-    <t>AllRegions</t>
-  </si>
-  <si>
-    <t>Pset_PD</t>
-  </si>
-  <si>
-    <t>Cset_Set</t>
-  </si>
-  <si>
-    <t>Cset_CD</t>
-  </si>
-  <si>
-    <t>Attrib_Cond</t>
-  </si>
-  <si>
-    <t>Val_Cond</t>
-  </si>
-  <si>
-    <t>~TFM_INS</t>
-  </si>
-  <si>
-    <t>ELC</t>
-  </si>
-  <si>
-    <t>COM_PKRSV</t>
-  </si>
-  <si>
-    <t>COM_PEAK</t>
-  </si>
-  <si>
-    <t>REG1</t>
   </si>
 </sst>
 </file>
@@ -838,12 +838,12 @@
   <sheetData>
     <row r="1" spans="1:1" ht="15">
       <c r="A1" t="s">
-        <v>8</v>
+        <v>18</v>
       </c>
     </row>
     <row r="2" spans="2:17" ht="15">
       <c r="B2" s="1" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="J2" s="2"/>
       <c r="K2" s="3"/>
@@ -856,68 +856,68 @@
     </row>
     <row r="3" spans="2:17" ht="15.75" thickBot="1">
       <c r="B3" s="4" t="s">
-        <v>9</v>
+        <v>19</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="F3" s="4" t="s">
-        <v>14</v>
+        <v>5</v>
       </c>
       <c r="G3" s="4" t="s">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="H3" s="5" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="I3" s="5" t="s">
-        <v>20</v>
+        <v>2</v>
       </c>
       <c r="J3" s="6" t="s">
         <v>3</v>
       </c>
       <c r="K3" s="6" t="s">
-        <v>2</v>
+        <v>20</v>
       </c>
       <c r="L3" s="6" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="M3" s="6" t="s">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="N3" s="6" t="s">
-        <v>5</v>
+        <v>14</v>
       </c>
       <c r="O3" s="6" t="s">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="P3" s="6" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="Q3" s="6" t="s">
-        <v>13</v>
+        <v>7</v>
       </c>
     </row>
     <row r="4" spans="4:16" ht="15">
       <c r="D4" s="7" t="s">
-        <v>19</v>
+        <v>9</v>
       </c>
       <c r="I4" s="8">
         <v>1</v>
       </c>
       <c r="P4" t="s">
-        <v>17</v>
+        <v>8</v>
       </c>
     </row>
     <row r="5" spans="4:16" ht="15">
       <c r="D5" s="7" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="E5">
         <v>2005</v>
@@ -926,21 +926,21 @@
         <v>0.05</v>
       </c>
       <c r="P5" t="s">
-        <v>17</v>
+        <v>8</v>
       </c>
     </row>
     <row r="6" spans="4:16" ht="15">
       <c r="D6" s="7" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="E6">
         <v>2020</v>
       </c>
       <c r="I6" s="11">
-        <v>0.20</v>
+        <v>0.30</v>
       </c>
       <c r="P6" t="s">
-        <v>17</v>
+        <v>8</v>
       </c>
     </row>
     <row r="7" spans="4:9" ht="15">

</xml_diff>